<commit_message>
scan: seg7 2026-06-22 21:29 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq8_2026-06-22.xlsx
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1070.841953716358</v>
+        <v>1080.841953716358</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>315</v>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>899.388167795476</v>
+        <v>909.388167795476</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>142</v>
@@ -1216,21 +1216,21 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>8039</v>
+        <v>6949</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>台虹</t>
+          <t>沛爾生醫-創</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>830.044794652198</v>
+        <v>828.7438295537238</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>153</v>
+        <v>886</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,16 +1241,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>56.77585605580573</v>
+        <v>71.96264451865591</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>22.08793750047158</v>
+        <v>29.41483975150739</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0.72011017013854</v>
+        <v>1.174382955372374</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.4628123150707406</v>
+        <v>27.18254583348319</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>6949</v>
+        <v>6901</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>沛爾生醫-創</t>
+          <t>鑽石投資</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>828.7438295537238</v>
+        <v>826.8867754245314</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>886</v>
+        <v>17.35</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,16 +1294,16 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>71.96264451865591</v>
+        <v>72.03774879379212</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>29.41483975150739</v>
+        <v>36.85090601315635</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>1.174382955372374</v>
+        <v>1.288677542453143</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1312,31 +1312,31 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>27.18254583348319</v>
+        <v>0.241105957525315</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>6901</v>
+        <v>8039</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>鑽石投資</t>
+          <t>台虹</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>826.8867754245314</v>
+        <v>810.044794652198</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>17.35</v>
+        <v>153</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,16 +1347,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>72.03774879379212</v>
+        <v>56.77585605580573</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>36.85090601315635</v>
+        <v>22.08793750047158</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>1.288677542453143</v>
+        <v>0.72011017013854</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -1365,11 +1365,11 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.241105957525315</v>
+        <v>0.4628123150707406</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2064,21 +2064,21 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6909</v>
+        <v>7827</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>漢康-KY創</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>673.0075949155932</v>
+        <v>667.4359359618011</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>55.9</v>
+        <v>159</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>61.68865815717073</v>
+        <v>55.42694233571278</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>19.80129909842692</v>
+        <v>23.88105427416988</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.7571252650656728</v>
+        <v>1.070799694736547</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.7884220096990924</v>
+        <v>0.2935415188147834</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, stronger_than_market, obv_uptrend, cci_momentum</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>7827</v>
+        <v>7714</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>漢康-KY創</t>
+          <t>創泓科技</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>667.4359359618011</v>
+        <v>666.3344356828675</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>159</v>
+        <v>132</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>55.42694233571278</v>
+        <v>54.67883113710729</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>23.88105427416988</v>
+        <v>23.04538649337943</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1.070799694736547</v>
+        <v>0.506115903103187</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.2935415188147834</v>
+        <v>0.0861404601625496</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>7714</v>
+        <v>6909</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>創泓科技</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>666.3344356828675</v>
+        <v>663.0075949155932</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>132</v>
+        <v>55.9</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>54.67883113710729</v>
+        <v>61.68865815717073</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>23.04538649337943</v>
+        <v>19.80129909842692</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.506115903103187</v>
+        <v>0.7571252650656728</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,11 +2213,11 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.0861404601625496</v>
+        <v>0.7884220096990924</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, stronger_than_market, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scan: seg7 2026-06-23 00:03 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq8_2026-06-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>65.53941580474768</v>
+        <v>65.53941578939164</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14.08558312912177</v>
+        <v>14.0855832782581</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>3.124808121510326</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>5.726838699930477</v>
+        <v>5.726838700651671</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -591,7 +591,7 @@
         <v/>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1127.78143009109</v>
+        <v>1127.781430091091</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>40.05</v>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>62.29553060734708</v>
+        <v>62.29553040050913</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>16.06335612174647</v>
+        <v>16.0633562090109</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.954375241811371</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.3340525494148201</v>
+        <v>0.3340525499093568</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>82.70526895458309</v>
+        <v>82.705268953607</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>56.15356066007343</v>
+        <v>56.15356067500338</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.294561870401536</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>50.78626233106689</v>
+        <v>50.78626233100505</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>64.6124946190953</v>
+        <v>64.61249464297514</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>40.40547901303975</v>
+        <v>40.40547901201923</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.80409818761825</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-1.135008262376795</v>
+        <v>-1.135008262479818</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>55.92908608257266</v>
+        <v>55.92908606427126</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>16.17834666101594</v>
+        <v>16.1783465031223</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.260385849884799</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>27.43942294530517</v>
+        <v>27.43942294942626</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>966.3115771791344</v>
+        <v>966.3115771791312</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>49.5</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>60.52424529368585</v>
+        <v>60.52424521715166</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>20.18463648775818</v>
+        <v>20.18463645012613</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.249711004982915</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.4502598620922589</v>
+        <v>0.450259862154078</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>71.55180234693373</v>
+        <v>71.55180158979235</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>17.91251986446619</v>
+        <v>17.91252017752273</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>2.209169120960922</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>2.612181980228874</v>
+        <v>2.612181992036776</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>60.36429056031709</v>
+        <v>60.36429053138892</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>22.99476762132414</v>
+        <v>22.99476737923556</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.9967047690751408</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.5384503807372401</v>
+        <v>0.5384503818705428</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>57.87268347945179</v>
+        <v>57.87268342944675</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>8.565402096045291</v>
+        <v>8.565401980362671</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.797460138376191</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.8000157175339941</v>
+        <v>0.8000157177812706</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>881.3486508729926</v>
+        <v>881.3486508729925</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>139</v>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>55.26169908397442</v>
+        <v>55.26169907763654</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>11.70043689525158</v>
+        <v>11.7004368965966</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>2.584528994940575</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>2.694166931591131</v>
+        <v>2.694166931900218</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>56.17900772746514</v>
+        <v>56.17900770861071</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>22.63485299023408</v>
+        <v>22.63485299830877</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.231887182263663</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>29.67550275759424</v>
+        <v>29.67550276068461</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>75.21922953458142</v>
+        <v>75.21922951439551</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>30.99631411417658</v>
+        <v>30.99631413673911</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>4.759921436431765</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.6750639150051677</v>
+        <v>0.6750639151081964</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>72.81655659836873</v>
+        <v>72.81655656558846</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>24.0888004030972</v>
+        <v>24.08880040331485</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.036625493860522</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>3.609650399355787</v>
+        <v>3.609650401725472</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>71.96264451865591</v>
+        <v>71.96264451494326</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>29.41483975150739</v>
+        <v>29.414839717208</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.174382955372374</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>27.18254583348319</v>
+        <v>27.18254583389537</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>72.03774879379212</v>
+        <v>72.03774859324403</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>36.85090601315635</v>
+        <v>36.85090614576939</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.288677542453143</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.241105957525315</v>
+        <v>0.2411059576798583</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>56.77585605580573</v>
+        <v>56.77585605057832</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>22.08793750047158</v>
+        <v>22.08793742974047</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.72011017013854</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.4628123150707406</v>
+        <v>0.4628123153283086</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>70.73825104810226</v>
+        <v>70.73825104068908</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>45.09811787178605</v>
+        <v>45.09811787312288</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.064199249198117</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>3.345247130384969</v>
+        <v>3.345247130549829</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>58.3926558217757</v>
+        <v>58.39265582639675</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>40.84830246858383</v>
+        <v>40.8483024435624</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.188813783444668</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-4.42211291515153</v>
+        <v>-4.422112914327268</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>60.66610626680457</v>
+        <v>60.66610624635464</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>25.41900634698354</v>
+        <v>25.41900629048462</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.800464692530777</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>2.332372952975227</v>
+        <v>2.332372953696453</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>58.91747297206508</v>
+        <v>58.91747287267873</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>33.12827533435173</v>
+        <v>33.12827552795318</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.7538579750174348</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-1.698124777149528</v>
+        <v>-1.698124776242865</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         <v>52.84481180660978</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>21.31423403999112</v>
+        <v>21.31423406669313</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>2.095219510608629</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>55.33585958156239</v>
+        <v>55.33585957843544</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>27.41086061028644</v>
+        <v>27.41086059759746</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.9886492997523362</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-2.452908067263746</v>
+        <v>-2.452908067098921</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>64.59190959429381</v>
+        <v>64.59190931504503</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>34.00606950311668</v>
+        <v>34.00606948579218</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.8233878643285483</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.3113181718849622</v>
+        <v>0.311318171998296</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>48.51930631514277</v>
+        <v>48.51930612853077</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>20.83701898442337</v>
+        <v>20.83701896198816</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.3920770726601247</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-1.742956603611957</v>
+        <v>-1.742956601345324</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>70.71443867068426</v>
+        <v>70.71443863971538</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>18.088740134527</v>
+        <v>18.08874001087502</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1.285757063097615</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>13.51436185592986</v>
+        <v>13.5143618610814</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>59.90082751704404</v>
+        <v>59.90082788541738</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>47.43078870497891</v>
+        <v>47.4307887025389</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.865379395097398</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.3542559727212192</v>
+        <v>0.3542559724636456</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>61.43996970325951</v>
+        <v>61.43996968810479</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>25.23654518245039</v>
+        <v>25.23654516143861</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>1.321342794334152</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-0.1628542545691673</v>
+        <v>-0.1628542545794717</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>58.88484999187227</v>
+        <v>58.88484997226321</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>14.40490346425581</v>
+        <v>14.40490344434206</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>2.199340296829913</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.0003687861347385</v>
+        <v>-0.0003687857226308</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>666.3344356828675</v>
+        <v>666.3344356828691</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>132</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>54.67883113710729</v>
+        <v>54.6788309216078</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>23.04538649337943</v>
+        <v>23.04538674204244</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.506115903103187</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.0861404601625496</v>
+        <v>0.0861404628413075</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>61.68865815717073</v>
+        <v>61.68865821967916</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>19.80129909842692</v>
+        <v>19.80129895353833</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.7571252650656728</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.7884220096990924</v>
+        <v>0.7884220095857626</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>661.4452813234014</v>
+        <v>661.4452813234016</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>386</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>62.49504204930312</v>
+        <v>62.49504174231156</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>29.63720720907401</v>
+        <v>29.63720753119228</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.48954814552421</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>4.441528867532453</v>
+        <v>4.44152888133835</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>648.6632391680655</v>
+        <v>648.6632391680656</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>135.5</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>60.89698249187427</v>
+        <v>60.89698233490566</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>29.14986424210636</v>
+        <v>29.14986433752845</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1.327843639926019</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.8224930621883315</v>
+        <v>0.8224930629095306</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>630.4080174310435</v>
+        <v>630.4080174310434</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>46.65</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>59.87027547436997</v>
+        <v>59.87027538448567</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>29.3198018321796</v>
+        <v>29.31980170715418</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.5096354683327952</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.0943100555137863</v>
+        <v>0.0943100555962155</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>53.45401389781811</v>
+        <v>53.45401384640675</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>25.77747461119767</v>
+        <v>25.77747452114154</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.6308660386242729</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.6202501348574732</v>
+        <v>-0.6202501344453704</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>69.6204293361062</v>
+        <v>69.62042935061569</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>43.90361435516697</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>5.06276613932242</v>
+        <v>5.062766138910312</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>65.01099320136322</v>
+        <v>65.01099317302777</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>28.35277190670049</v>
+        <v>28.35277190166713</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.7295667084716324</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.0842639456011236</v>
+        <v>-0.08426394539508129</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>598.5844702026598</v>
+        <v>598.5844702026599</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>321</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>55.54820304584335</v>
+        <v>55.54820293223525</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>36.82782131945735</v>
+        <v>36.82782133229556</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.4092656219194371</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>2.621554466486423</v>
+        <v>2.621554469165193</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>52.63360728914351</v>
+        <v>52.63360731049897</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>30.30429525410425</v>
+        <v>30.30429527953677</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.5159382694264999</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-4.761208923049487</v>
+        <v>-4.761208922946434</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>54.56550134762211</v>
+        <v>54.56550140815041</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>23.84284775585728</v>
+        <v>23.84284791858276</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>2.001819203760846</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.0162998289390034</v>
+        <v>0.0162998288771855</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>57.2575022072945</v>
+        <v>57.25750208876467</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>9.73637492955784</v>
+        <v>9.736374940217589</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1.063996797820855</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.3667535222185266</v>
+        <v>0.3667535225070085</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>50.67362837693793</v>
+        <v>50.6736269724751</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>29.12310805168478</v>
+        <v>29.12310925320003</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>9.60196456241664</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-2.800574221496936</v>
+        <v>-2.800574200891138</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>48.86918602877905</v>
+        <v>48.86918603003997</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>24.28418617701989</v>
+        <v>24.28418616875807</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.408551454363652</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-118.831175378236</v>
+        <v>-118.8311753792662</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>52.42601263843648</v>
+        <v>52.42601263615424</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>8.863121571753698</v>
+        <v>8.863121668639701</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.9811173122887236</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.6726637701111772</v>
+        <v>0.6726637703172298</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>48.79921726095386</v>
+        <v>48.79921721578451</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>7.758144818757813</v>
+        <v>7.758144810984413</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.9646122528243534</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.0262058056861859</v>
+        <v>0.0262058057686112</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>34.55390107253774</v>
+        <v>34.55390057626508</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>18.90873051819294</v>
+        <v>18.90873065462169</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.937674307815006</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.5699170780031777</v>
+        <v>-0.5699170759426015</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>63.25570999644501</v>
+        <v>63.25571005911765</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>19.9254854335542</v>
+        <v>19.92548549000606</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>2.611020156785313</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.199355079337954</v>
+        <v>0.1993550792761358</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>49.95822080318814</v>
+        <v>49.95822084923119</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>16.39247691598555</v>
+        <v>16.39247694071452</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.922282794345022</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.2606198988803281</v>
+        <v>-0.260619899230634</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.32866759768103</v>
+        <v>50.32866757947092</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>20.47920390179484</v>
+        <v>20.47920387972108</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.9083102235495534</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-1.053411422646263</v>
+        <v>-1.053411413270766</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>52.0760053928479</v>
+        <v>52.07600504738843</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>17.53309812075693</v>
+        <v>17.53309812132323</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.4857500439517975</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-5.903995370529053</v>
+        <v>-5.903995371044211</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>50.28141551441858</v>
+        <v>50.28141550416476</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>11.38509597145553</v>
+        <v>11.38509593729336</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.5005233762158769</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.905593382875173</v>
+        <v>-0.9055933836993368</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>45.8888336373936</v>
+        <v>45.88883356389442</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>17.81052985736669</v>
+        <v>17.81052988165184</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6288692553880514</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.89356835314342</v>
+        <v>-0.8935683525252696</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>50.06794510754226</v>
+        <v>50.06794521693841</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>6.787441905764631</v>
+        <v>6.787441947119889</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.8024135897507904</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.114078280650044</v>
+        <v>0.1140782804439905</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>437.0047924280298</v>
+        <v>437.0047924280299</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>77.8</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>36.59609347795149</v>
+        <v>36.59609281455537</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>23.61185707125083</v>
+        <v>23.61185742186349</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.515367143515857</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.0717944048294071</v>
+        <v>0.0717944059627135</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>40.14267525458595</v>
+        <v>40.14267503058294</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>20.13037695449002</v>
+        <v>20.1303769695165</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>2.092737652041975</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.0578297818000626</v>
+        <v>0.0578297819649089</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>37.89052299112909</v>
+        <v>37.89052287193498</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>27.10871826457877</v>
+        <v>27.10871817477961</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.5707374734817302</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-9.385201005223593</v>
+        <v>-9.38520100110242</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>44.99872099221256</v>
+        <v>44.99872105395979</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>16.3566754971276</v>
+        <v>16.35667559454314</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.5549157930599485</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>50.34493338573455</v>
+        <v>50.34493339245611</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>17.27666665797279</v>
+        <v>17.2766667517978</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>1.799574560870713</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-2.201767910762873</v>
+        <v>-2.201767910680454</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>48.70281130584146</v>
+        <v>48.7028113670485</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>20.60069553684024</v>
+        <v>20.60069561740938</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.3147217342463461</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.5399927611570694</v>
+        <v>-0.5399927612394884</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>44.03502726589837</v>
+        <v>44.03502726416852</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>16.56019874239513</v>
+        <v>16.56019873504343</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.140711668229609</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>9.099274561333189</v>
+        <v>9.099274563084748</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>56.228634375814</v>
+        <v>56.22863428421953</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>12.85149333118437</v>
+        <v>12.85149320547774</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.7270043206102228</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>1.578746707336482</v>
+        <v>1.578746707851607</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>401.100055887049</v>
+        <v>401.1000558870491</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>128</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>44.7361196917019</v>
+        <v>44.73611971020996</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>5.361166064081067</v>
+        <v>5.36116605625589</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>2.422589797470218</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-1.071986065501019</v>
+        <v>-1.071986065191926</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>400.6012578441249</v>
+        <v>400.6012578441255</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>126.5</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>51.56033095601126</v>
+        <v>51.56033112730417</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>21.65111587151888</v>
+        <v>21.65111588490624</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.5085604670159811</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>46.09944799187934</v>
+        <v>46.09944795552155</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>12.7193931393145</v>
+        <v>12.71939316089449</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.7963255482381917</v>
@@ -4159,7 +4159,7 @@
         <v>50.10642352974052</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>19.41957782444251</v>
+        <v>19.41957783804279</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>1.094453660093672</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.1896182550762042</v>
+        <v>0.1896182554031962</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>370.4130003607813</v>
+        <v>370.4130003607814</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>63.4</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>45.92208379257372</v>
+        <v>45.92208369752853</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>20.72283982141096</v>
+        <v>20.72283991290439</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.3423057790707131</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.5995025336167696</v>
+        <v>-0.5995025331016286</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>42.54312097936246</v>
+        <v>42.5431211353528</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>14.35470045615136</v>
+        <v>14.35470049169649</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.2740705490452679</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.1229910272085863</v>
+        <v>0.1229910262813271</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>51.63591259256456</v>
+        <v>51.6359126381706</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>27.84964517027803</v>
+        <v>27.84964520832503</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5748077876889851</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-2.054718710938713</v>
+        <v>-2.05471871145386</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>349.8102881042452</v>
+        <v>349.8102881042451</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>95.40000000000001</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>37.43647068716717</v>
+        <v>37.43647065798573</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>22.32291334290928</v>
+        <v>22.3229133917388</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.9732468373371664</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-1.087510398821681</v>
+        <v>-1.087510399233792</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>42.4930940640572</v>
+        <v>42.493094256469</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>13.15285304042637</v>
+        <v>13.15285315176261</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.5138777370736521</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>43.8053760443205</v>
+        <v>43.80537609572517</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>14.81325982785105</v>
+        <v>14.81325983174465</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.8952870050360661</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-3.299727576521289</v>
+        <v>-3.299727576109164</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>336.183528234572</v>
+        <v>336.1835282345717</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>162.5</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>52.18835169667001</v>
+        <v>52.18835165630126</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>21.53210478487348</v>
+        <v>21.53210475556737</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.5795081489397166</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.8641927099165342</v>
+        <v>0.8641927097105027</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>53.80407853471839</v>
+        <v>53.80407892275137</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>13.43381818115378</v>
+        <v>13.43381821333766</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.5992270747479266</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.3814375528294385</v>
+        <v>0.3814375526233619</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>44.88039602803669</v>
+        <v>44.88039603034152</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>12.4085366913884</v>
+        <v>12.40853668243381</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.3847901495692781</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.8204996969755651</v>
+        <v>0.820499697696718</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>49.55380986321912</v>
+        <v>49.55380982312543</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.48795102674115</v>
+        <v>14.4879507898148</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.6939034297001327</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.9809704387780532</v>
+        <v>-0.9809704374386472</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>324.6352125145155</v>
+        <v>324.6352125145161</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>77.59999999999999</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>36.13885234746732</v>
+        <v>36.13885232123426</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>25.06356401839511</v>
+        <v>25.06356399042515</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>1.235248916813766</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.4836615934563927</v>
+        <v>-0.4836615933533592</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>36.57670047329545</v>
+        <v>36.57670061055075</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>23.74349506359022</v>
+        <v>23.74349505585824</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.121913241120369</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.2560651495362525</v>
+        <v>0.2560651495156514</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>315.0832149497721</v>
+        <v>315.0832149497715</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>101</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>53.55518297010312</v>
+        <v>53.55518288964359</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>20.44529666174306</v>
+        <v>20.44529672399069</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>1.425380245004285</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.8918850645285517</v>
+        <v>0.8918850648376404</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>48.35613041808492</v>
+        <v>48.35613021545147</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>14.2259371256239</v>
+        <v>14.22593718433371</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.7143605197950931</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.3610642212091439</v>
+        <v>-0.3610642206115808</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>49.19357979906669</v>
+        <v>49.19357974522927</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>13.4588723588169</v>
+        <v>13.45887237517531</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.4385209546499391</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.7553262681208945</v>
+        <v>-0.7553262672966641</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>312.663494418786</v>
+        <v>312.6634944187862</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>126</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>50.80731198963056</v>
+        <v>50.8073119965563</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>6.615636143309695</v>
+        <v>6.615636106534089</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.6796947814292533</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.140576755084854</v>
+        <v>-0.1405767551878662</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>45.85265060183961</v>
+        <v>45.8526509067259</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>12.33302096109692</v>
+        <v>12.33302097877633</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.8024665874823516</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.0583851760277486</v>
+        <v>-0.0583851763059266</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>49.48041574068085</v>
+        <v>49.48041585347485</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>21.30039897189609</v>
+        <v>21.30039885049917</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.5757675988618267</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.6223702488953147</v>
+        <v>0.6223702477001793</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>294.9237281042291</v>
+        <v>294.9237281042281</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>81.8</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>42.65663365627633</v>
+        <v>42.65663361257544</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>14.74411284932972</v>
+        <v>14.74411289410426</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.6107883314869827</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.9704984866731324</v>
+        <v>-0.9704984857458716</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>51.85172468705309</v>
+        <v>51.85172469722127</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>6.713896286956341</v>
+        <v>6.713896339004802</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.9392068790509556</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.1255403715868781</v>
+        <v>0.1255403715250622</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>50.70239242567776</v>
+        <v>50.70239241451672</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>6.891631615488098</v>
+        <v>6.891631521879737</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.3642950618635472</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.2523962860722427</v>
+        <v>0.2523962861443622</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>42.44541923199612</v>
+        <v>42.44541909981378</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>16.85769468694459</v>
+        <v>16.85769462865148</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.5101260824749427</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.0496003012098031</v>
+        <v>-0.0496003011376826</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>273.1727491073011</v>
+        <v>273.1727491073012</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>32</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>53.31316326029391</v>
+        <v>53.31316334405586</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>16.51680670590167</v>
+        <v>16.51680681484895</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.041311498919932</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.1358785532114742</v>
+        <v>0.135878553314504</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>270.1215532354501</v>
+        <v>270.1215532354503</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>125.5</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>43.93043415709543</v>
+        <v>43.93043399314701</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>16.66136635298323</v>
+        <v>16.66136629688741</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.471410791824543</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-1.193626239604751</v>
+        <v>-1.193626238059307</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>38.30257221625779</v>
+        <v>38.30257217599421</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>21.95696342944745</v>
+        <v>21.95696344544703</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.4234297774058224</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-2.046182092734957</v>
+        <v>-2.046182092631943</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>47.15742841112933</v>
+        <v>47.15742840173273</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>17.7512969662387</v>
+        <v>17.75129692963017</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.4572236535207403</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.3428153363164785</v>
+        <v>0.3428153364195392</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5746,7 +5746,7 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>35.90940265786756</v>
+        <v>35.90940264087642</v>
       </c>
       <c r="I100" s="2" t="n">
         <v>30.44031735373938</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>1.093159551285226</v>
+        <v>1.09315955130582</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>260.009984829291</v>
+        <v>260.0099848292908</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>864</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>50.68309809850406</v>
+        <v>50.68309808957587</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>14.60048464642928</v>
+        <v>14.60048448798617</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>1.170924787330161</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-2.193561408449039</v>
+        <v>-2.193561407748417</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>247.0987240118589</v>
+        <v>247.0987240118588</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>33</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.53466659174671</v>
+        <v>41.53466695183588</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>10.38524009751096</v>
+        <v>10.3852400910298</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>1.372148400481047</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0031018644713013</v>
+        <v>0.0031018642652469</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>38.02470556686635</v>
+        <v>38.02470540178611</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>20.63882721924165</v>
+        <v>20.63882754314813</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.7409797488891229</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.2817803578476974</v>
+        <v>0.2817803582907199</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5944,7 +5944,7 @@
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>245.6179135136154</v>
+        <v>245.6179135136144</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>233</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>39.84368585710199</v>
+        <v>39.84368582714896</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>27.42235368594513</v>
+        <v>27.42235370626345</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>1.381890834948984</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-2.496772082004131</v>
+        <v>-2.496772082210236</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>42.43995479889795</v>
+        <v>42.43995455959707</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>15.62205800843197</v>
+        <v>15.62205799569434</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.489022309856659</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>35.22825300758657</v>
+        <v>35.2282463082099</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>17.82677782864999</v>
+        <v>17.82677679730355</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.6807308634121423</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.1173076292896997</v>
+        <v>-0.1173076251685378</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>51.39407745176673</v>
+        <v>51.39407743736668</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>23.99055270485378</v>
+        <v>23.99055270575149</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.4387346723604955</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>47.38656670620628</v>
+        <v>47.38656649761595</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>18.52522282287528</v>
+        <v>18.52522318093171</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.272322182786586</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0817736004429495</v>
+        <v>0.0817736006490099</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>40.73484829346652</v>
+        <v>40.73484809103385</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>17.55611649638823</v>
+        <v>17.55611644095139</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.6860105144286046</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.6487330630657198</v>
+        <v>-0.6487330616232923</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>41.41650040164578</v>
+        <v>41.41650038035947</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>22.56176257626873</v>
+        <v>22.56176260963538</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.7812924426148683</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>42.88622439463482</v>
+        <v>42.8862243913179</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>15.84542103785307</v>
+        <v>15.84542111280202</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.7403640116271107</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.9785327905661836</v>
+        <v>-0.97853279050433</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>44.28980985596638</v>
+        <v>44.28980976969418</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>15.2381057289673</v>
+        <v>15.23810570854576</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.5627322706185505</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0147171217449512</v>
+        <v>0.0147171217861583</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>47.207182245479</v>
+        <v>47.20718204602086</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>11.08699777379715</v>
+        <v>11.08699790243511</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.6350893367821685</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0723040870386694</v>
+        <v>0.0723040873477486</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>51.93558382188857</v>
+        <v>51.93558380936884</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>16.35073702216502</v>
+        <v>16.35073706156415</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.9912661507575627</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.6176966859886703</v>
+        <v>-0.6176966858650383</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>37.54669960548357</v>
+        <v>37.5466996792243</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>16.95227765698967</v>
+        <v>16.95227795821262</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.5548128590195885</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.5186236693596429</v>
+        <v>-0.518623668226327</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>22.8860787564861</v>
+        <v>22.88607879033405</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>19.76810346478903</v>
+        <v>19.76810344284568</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.67209701350892</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.1010756334848535</v>
+        <v>-0.101075633299402</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>49.25939466292439</v>
+        <v>49.25939469697882</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>14.51911459738441</v>
+        <v>14.51911463951046</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.7236481883907269</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>2.836014530921805</v>
+        <v>2.836014529891518</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>39.88516649958735</v>
+        <v>39.88516418565724</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>31.5995439208532</v>
+        <v>31.59954501884643</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>1.131575738605866</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.0954545263312462</v>
+        <v>0.0954545386741192</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>49.9220270177262</v>
+        <v>49.92202709560357</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>5.917758627051258</v>
+        <v>5.917758611031175</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.4714774659772882</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.2150610343363386</v>
+        <v>0.2150610338418037</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>27.35587972137277</v>
+        <v>27.3558800058688</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>50.39218148929477</v>
+        <v>50.39218143100182</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.5961442632433621</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>1.300112664939156</v>
+        <v>1.300112665248253</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,7 +6912,7 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>36.21066639002928</v>
+        <v>36.21066639638281</v>
       </c>
       <c r="I122" s="2" t="n">
         <v>20.89995061441329</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.4075506922579559</v>
+        <v>-0.4075506923197663</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>41.92846547331165</v>
+        <v>41.92846538144149</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>16.84162555987976</v>
+        <v>16.84162565769788</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.7778136964713251</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.2236692246028502</v>
+        <v>0.2236692246955689</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>41.01078492707575</v>
+        <v>41.01078483398764</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>12.68448449415814</v>
+        <v>12.6844844554728</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.8262117755659648</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.1085622701272415</v>
+        <v>-0.1085622700036097</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>43.59213547075326</v>
+        <v>43.59213535661334</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>16.91612053647028</v>
+        <v>16.91612060627184</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.9314210615928148</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.1425580567565704</v>
+        <v>-0.1425580565917258</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>

</xml_diff>